<commit_message>
Auto-load default lecture data on startup and group fields into 5 sections
</commit_message>
<xml_diff>
--- a/sample/DULIEU_BaiGiang.xlsx
+++ b/sample/DULIEU_BaiGiang.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dữ liệu bài giảng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu bài giảng" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dữ liệu bài giảng'!$A$1:$B$49</definedName>
@@ -719,63 +719,63 @@
     <author>Mẫu bài giảng</author>
   </authors>
   <commentList>
-    <comment ref="B12" authorId="0" shapeId="0">
+    <comment ref="B11" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
 Phần mềm sẽ tự sinh ra "Ngày 07 tháng 4 năm 2026" khi trộn.</t>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0">
+    <comment ref="C11" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
 Phần mềm sẽ tự sinh ra "Ngày 07 tháng 4 năm 2026" khi trộn.</t>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
+    <comment ref="B12" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C13" authorId="0" shapeId="0">
+    <comment ref="C12" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B13" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C14" authorId="0" shapeId="0">
+    <comment ref="C13" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B22" authorId="0" shapeId="0">
+    <comment ref="B20" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
 Phần mềm sẽ tự sinh ra "Ngày 07 tháng 4 năm 2026" khi trộn.</t>
       </text>
     </comment>
-    <comment ref="C22" authorId="0" shapeId="0">
+    <comment ref="C20" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
 Phần mềm sẽ tự sinh ra "Ngày 07 tháng 4 năm 2026" khi trộn.</t>
       </text>
     </comment>
-    <comment ref="B26" authorId="0" shapeId="0">
+    <comment ref="B23" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
@@ -785,7 +785,7 @@
 Trang bìa chỉ lấy tháng và năm của ô này.</t>
       </text>
     </comment>
-    <comment ref="C26" authorId="0" shapeId="0">
+    <comment ref="C23" authorId="0" shapeId="0">
       <text>
         <t>Nhập theo dạng ngày/tháng/năm, ví dụ 07/04/2026.
 Ô này là ngày thật của Excel, không phải chuỗi chữ.
@@ -795,160 +795,190 @@
 Trang bìa chỉ lấy tháng và năm của ô này.</t>
       </text>
     </comment>
-    <comment ref="B27" authorId="0" shapeId="0">
+    <comment ref="B24" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C27" authorId="0" shapeId="0">
+    <comment ref="C24" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B28" authorId="0" shapeId="0">
+    <comment ref="B25" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C28" authorId="0" shapeId="0">
+    <comment ref="C25" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B29" authorId="0" shapeId="0">
+    <comment ref="B26" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C29" authorId="0" shapeId="0">
+    <comment ref="C26" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B30" authorId="0" shapeId="0">
+    <comment ref="B27" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C30" authorId="0" shapeId="0">
+    <comment ref="C27" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B31" authorId="0" shapeId="0">
+    <comment ref="B28" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C31" authorId="0" shapeId="0">
+    <comment ref="C28" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B33" authorId="0" shapeId="0">
+    <comment ref="B30" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C33" authorId="0" shapeId="0">
+    <comment ref="C30" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B34" authorId="0" shapeId="0">
+    <comment ref="B31" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C34" authorId="0" shapeId="0">
+    <comment ref="C31" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B35" authorId="0" shapeId="0">
+    <comment ref="B32" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C35" authorId="0" shapeId="0">
+    <comment ref="C32" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B36" authorId="0" shapeId="0">
+    <comment ref="B33" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C36" authorId="0" shapeId="0">
+    <comment ref="C33" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B38" authorId="0" shapeId="0">
+    <comment ref="B35" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C38" authorId="0" shapeId="0">
+    <comment ref="C35" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="B39" authorId="0" shapeId="0">
+    <comment ref="B36" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C39" authorId="0" shapeId="0">
+    <comment ref="C36" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
+    <comment ref="B39" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
+    <comment ref="C39" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
+    <comment ref="B40" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
+    <comment ref="C40" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
+    <comment ref="B41" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
+    <comment ref="C41" authorId="0" shapeId="0">
+      <text>
+        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
+      </text>
+    </comment>
     <comment ref="B42" authorId="0" shapeId="0">
       <text>
         <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
@@ -989,44 +1019,14 @@
         <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
       </text>
     </comment>
-    <comment ref="B46" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
-    <comment ref="C46" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
-    <comment ref="B47" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
-    <comment ref="C47" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
     <comment ref="B48" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
-    <comment ref="C48" authorId="0" shapeId="0">
-      <text>
-        <t>Chỉ nhập con số, ví dụ 90. Dấu ngoặc và chữ "phút" đã có sẵn trong file Word mẫu.</t>
-      </text>
-    </comment>
-    <comment ref="B51" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
 Không tách sang ô khác, không dùng dấu | để ngăn cách.</t>
       </text>
     </comment>
-    <comment ref="C51" authorId="0" shapeId="0">
+    <comment ref="C48" authorId="0" shapeId="0">
       <text>
         <t>Trường nhiều dòng.
 Bấm Alt + Enter để xuống dòng ngay trong ô này, mỗi gạch đầu dòng một dòng.
@@ -1326,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y63"/>
+  <dimension ref="A1:Y60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1648,17 +1648,17 @@
     <row r="9">
       <c r="A9" s="93" t="inlineStr">
         <is>
-          <t>Cấp bậc, học vị người phê duyệt</t>
+          <t>Cấp bậc, học vị, họ tên người phê duyệt</t>
         </is>
       </c>
       <c r="B9" s="94" t="inlineStr">
         <is>
-          <t>Đại tá, TS</t>
+          <t>Đại tá, TS Đào Mạnh Hùng</t>
         </is>
       </c>
       <c r="C9" s="94" t="inlineStr">
         <is>
-          <t>Đại tá, TS</t>
+          <t>Đại tá, TS Đào Mạnh Hùng</t>
         </is>
       </c>
       <c r="D9" s="94" t="n"/>
@@ -1687,17 +1687,17 @@
     <row r="10">
       <c r="A10" s="93" t="inlineStr">
         <is>
-          <t>Họ tên người phê duyệt</t>
+          <t>Địa điểm phê duyệt</t>
         </is>
       </c>
       <c r="B10" s="94" t="inlineStr">
         <is>
-          <t>Đào Mạnh Hùng</t>
+          <t>Văn phòng khoa</t>
         </is>
       </c>
       <c r="C10" s="94" t="inlineStr">
         <is>
-          <t>Đào Mạnh Hùng</t>
+          <t>Văn phòng khoa</t>
         </is>
       </c>
       <c r="D10" s="94" t="n"/>
@@ -1726,18 +1726,14 @@
     <row r="11">
       <c r="A11" s="93" t="inlineStr">
         <is>
-          <t>Địa điểm phê duyệt</t>
-        </is>
-      </c>
-      <c r="B11" s="94" t="inlineStr">
-        <is>
-          <t>Văn phòng khoa</t>
-        </is>
-      </c>
-      <c r="C11" s="94" t="inlineStr">
-        <is>
-          <t>Văn phòng khoa</t>
-        </is>
+          <t>Ngày phê duyệt</t>
+        </is>
+      </c>
+      <c r="B11" s="95" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C11" s="95" t="n">
+        <v>46119</v>
       </c>
       <c r="D11" s="94" t="n"/>
       <c r="E11" s="94" t="n"/>
@@ -1765,14 +1761,20 @@
     <row r="12">
       <c r="A12" s="93" t="inlineStr">
         <is>
-          <t>Ngày phê duyệt</t>
-        </is>
-      </c>
-      <c r="B12" s="95" t="n">
-        <v>46119</v>
-      </c>
-      <c r="C12" s="95" t="n">
-        <v>46119</v>
+          <t>Nhận xét phần nội dung bài giảng</t>
+        </is>
+      </c>
+      <c r="B12" s="94" t="inlineStr">
+        <is>
+          <t>- Nội dung bài giảng phù hợp với mục đích, yêu cầu, chuẩn đầu ra, đề cương học phần trang bị điển hình súng bộ binh;
+- Cấu trúc bài giảng rõ ràng, đảm bảo tính khoa học, logic; sử dụng tài liệu chính, tham khảo cập nhật, phù hợp.</t>
+        </is>
+      </c>
+      <c r="C12" s="94" t="inlineStr">
+        <is>
+          <t>- Nội dung bài giảng phù hợp với mục đích, yêu cầu, chuẩn đầu ra, đề cương học phần trang bị điển hình súng bộ binh;
+- Cấu trúc bài giảng rõ ràng, đảm bảo tính khoa học, logic; sử dụng tài liệu chính, tham khảo cập nhật, phù hợp.</t>
+        </is>
       </c>
       <c r="D12" s="94" t="n"/>
       <c r="E12" s="94" t="n"/>
@@ -1800,19 +1802,19 @@
     <row r="13">
       <c r="A13" s="93" t="inlineStr">
         <is>
-          <t>Nhận xét phần nội dung bài giảng</t>
+          <t>Nhận xét phần thực hành giảng bài</t>
         </is>
       </c>
       <c r="B13" s="94" t="inlineStr">
         <is>
-          <t>- Nội dung bài giảng phù hợp với mục đích, yêu cầu, chuẩn đầu ra, đề cương học phần trang bị điển hình súng bộ binh;
-- Cấu trúc bài giảng rõ ràng, đảm bảo tính khoa học, logic; sử dụng tài liệu chính, tham khảo cập nhật, phù hợp.</t>
+          <t>- Phù hợp với đối tượng, bảo đảm nội dung và thời gian;
+- Phương pháp giảng dạy phù hợp, có kế hoạch tổ chức lớp học, phân chia thời gian, tương tác với người học; học liệu đầy đủ.</t>
         </is>
       </c>
       <c r="C13" s="94" t="inlineStr">
         <is>
-          <t>- Nội dung bài giảng phù hợp với mục đích, yêu cầu, chuẩn đầu ra, đề cương học phần trang bị điển hình súng bộ binh;
-- Cấu trúc bài giảng rõ ràng, đảm bảo tính khoa học, logic; sử dụng tài liệu chính, tham khảo cập nhật, phù hợp.</t>
+          <t>- Phù hợp với đối tượng, bảo đảm nội dung và thời gian;
+- Phương pháp giảng dạy phù hợp, có kế hoạch tổ chức lớp học, phân chia thời gian, tương tác với người học; học liệu đầy đủ.</t>
         </is>
       </c>
       <c r="D13" s="94" t="n"/>
@@ -1841,19 +1843,17 @@
     <row r="14">
       <c r="A14" s="93" t="inlineStr">
         <is>
-          <t>Nhận xét phần thực hành giảng bài</t>
+          <t>Kết luận phê duyệt</t>
         </is>
       </c>
       <c r="B14" s="94" t="inlineStr">
         <is>
-          <t>- Phù hợp với đối tượng, bảo đảm nội dung và thời gian;
-- Phương pháp giảng dạy phù hợp, có kế hoạch tổ chức lớp học, phân chia thời gian, tương tác với người học; học liệu đầy đủ.</t>
+          <t>Đồng ý phần nội dung, phần thực hành giảng bài.</t>
         </is>
       </c>
       <c r="C14" s="94" t="inlineStr">
         <is>
-          <t>- Phù hợp với đối tượng, bảo đảm nội dung và thời gian;
-- Phương pháp giảng dạy phù hợp, có kế hoạch tổ chức lớp học, phân chia thời gian, tương tác với người học; học liệu đầy đủ.</t>
+          <t>Đồng ý phần nội dung, phần thực hành giảng bài.</t>
         </is>
       </c>
       <c r="D14" s="94" t="n"/>
@@ -1880,58 +1880,58 @@
       <c r="Y14" s="94" t="n"/>
     </row>
     <row r="15" thickBot="1">
-      <c r="A15" s="93" t="inlineStr">
-        <is>
-          <t>Kết luận phê duyệt</t>
-        </is>
-      </c>
-      <c r="B15" s="94" t="inlineStr">
-        <is>
-          <t>Đồng ý phần nội dung, phần thực hành giảng bài.</t>
-        </is>
-      </c>
-      <c r="C15" s="94" t="inlineStr">
-        <is>
-          <t>Đồng ý phần nội dung, phần thực hành giảng bài.</t>
-        </is>
-      </c>
-      <c r="D15" s="94" t="n"/>
-      <c r="E15" s="94" t="n"/>
-      <c r="F15" s="94" t="n"/>
-      <c r="G15" s="94" t="n"/>
-      <c r="H15" s="94" t="n"/>
-      <c r="I15" s="94" t="n"/>
-      <c r="J15" s="94" t="n"/>
-      <c r="K15" s="94" t="n"/>
-      <c r="L15" s="94" t="n"/>
-      <c r="M15" s="94" t="n"/>
-      <c r="N15" s="94" t="n"/>
-      <c r="O15" s="94" t="n"/>
-      <c r="P15" s="94" t="n"/>
-      <c r="Q15" s="94" t="n"/>
-      <c r="R15" s="94" t="n"/>
-      <c r="S15" s="94" t="n"/>
-      <c r="T15" s="94" t="n"/>
-      <c r="U15" s="94" t="n"/>
-      <c r="V15" s="94" t="n"/>
-      <c r="W15" s="94" t="n"/>
-      <c r="X15" s="94" t="n"/>
-      <c r="Y15" s="94" t="n"/>
+      <c r="A15" s="96" t="inlineStr">
+        <is>
+          <t>Chức vụ người thông qua</t>
+        </is>
+      </c>
+      <c r="B15" s="97" t="inlineStr">
+        <is>
+          <t>CHỦ NHIỆM KHOA</t>
+        </is>
+      </c>
+      <c r="C15" s="97" t="inlineStr">
+        <is>
+          <t>CHỦ NHIỆM KHOA</t>
+        </is>
+      </c>
+      <c r="D15" s="97" t="n"/>
+      <c r="E15" s="97" t="n"/>
+      <c r="F15" s="97" t="n"/>
+      <c r="G15" s="97" t="n"/>
+      <c r="H15" s="97" t="n"/>
+      <c r="I15" s="97" t="n"/>
+      <c r="J15" s="97" t="n"/>
+      <c r="K15" s="97" t="n"/>
+      <c r="L15" s="97" t="n"/>
+      <c r="M15" s="97" t="n"/>
+      <c r="N15" s="97" t="n"/>
+      <c r="O15" s="97" t="n"/>
+      <c r="P15" s="97" t="n"/>
+      <c r="Q15" s="97" t="n"/>
+      <c r="R15" s="97" t="n"/>
+      <c r="S15" s="97" t="n"/>
+      <c r="T15" s="97" t="n"/>
+      <c r="U15" s="97" t="n"/>
+      <c r="V15" s="97" t="n"/>
+      <c r="W15" s="97" t="n"/>
+      <c r="X15" s="97" t="n"/>
+      <c r="Y15" s="97" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="96" t="inlineStr">
         <is>
-          <t>Chức vụ người thông qua</t>
+          <t>Cấp bậc, học vị, họ tên người thông qua</t>
         </is>
       </c>
       <c r="B16" s="97" t="inlineStr">
         <is>
-          <t>CHỦ NHIỆM KHOA</t>
+          <t>Đại tá, TS Đào Mạnh Hùng</t>
         </is>
       </c>
       <c r="C16" s="97" t="inlineStr">
         <is>
-          <t>CHỦ NHIỆM KHOA</t>
+          <t>Đại tá, TS Đào Mạnh Hùng</t>
         </is>
       </c>
       <c r="D16" s="97" t="n"/>
@@ -1960,17 +1960,17 @@
     <row r="17">
       <c r="A17" s="96" t="inlineStr">
         <is>
-          <t>Cấp bậc, học vị người thông qua</t>
+          <t>Phương pháp thông qua</t>
         </is>
       </c>
       <c r="B17" s="97" t="inlineStr">
         <is>
-          <t>Đại tá, TS</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C17" s="97" t="inlineStr">
         <is>
-          <t>Đại tá, TS</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="D17" s="97" t="n"/>
@@ -1999,17 +1999,17 @@
     <row r="18">
       <c r="A18" s="96" t="inlineStr">
         <is>
-          <t>Họ tên người thông qua</t>
+          <t>Địa điểm thông qua</t>
         </is>
       </c>
       <c r="B18" s="97" t="inlineStr">
         <is>
-          <t>Đào Mạnh Hùng</t>
+          <t>H2.10</t>
         </is>
       </c>
       <c r="C18" s="97" t="inlineStr">
         <is>
-          <t>Đào Mạnh Hùng</t>
+          <t>H2.10</t>
         </is>
       </c>
       <c r="D18" s="97" t="n"/>
@@ -2038,17 +2038,17 @@
     <row r="19">
       <c r="A19" s="96" t="inlineStr">
         <is>
-          <t>Phương pháp thông qua</t>
+          <t>Giờ thông qua</t>
         </is>
       </c>
       <c r="B19" s="97" t="inlineStr">
         <is>
-          <t>Báo cáo</t>
+          <t>08h00</t>
         </is>
       </c>
       <c r="C19" s="97" t="inlineStr">
         <is>
-          <t>Báo cáo</t>
+          <t>08h00</t>
         </is>
       </c>
       <c r="D19" s="97" t="n"/>
@@ -2077,18 +2077,14 @@
     <row r="20">
       <c r="A20" s="96" t="inlineStr">
         <is>
-          <t>Địa điểm thông qua</t>
-        </is>
-      </c>
-      <c r="B20" s="97" t="inlineStr">
-        <is>
-          <t>H2.10</t>
-        </is>
-      </c>
-      <c r="C20" s="97" t="inlineStr">
-        <is>
-          <t>H2.10</t>
-        </is>
+          <t>Ngày thông qua</t>
+        </is>
+      </c>
+      <c r="B20" s="98" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C20" s="98" t="n">
+        <v>46118</v>
       </c>
       <c r="D20" s="97" t="n"/>
       <c r="E20" s="97" t="n"/>
@@ -2114,94 +2110,94 @@
       <c r="Y20" s="97" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="96" t="inlineStr">
-        <is>
-          <t>Giờ thông qua</t>
-        </is>
-      </c>
-      <c r="B21" s="97" t="inlineStr">
-        <is>
-          <t>08h00</t>
-        </is>
-      </c>
-      <c r="C21" s="97" t="inlineStr">
-        <is>
-          <t>08h00</t>
-        </is>
-      </c>
-      <c r="D21" s="97" t="n"/>
-      <c r="E21" s="97" t="n"/>
-      <c r="F21" s="97" t="n"/>
-      <c r="G21" s="97" t="n"/>
-      <c r="H21" s="97" t="n"/>
-      <c r="I21" s="97" t="n"/>
-      <c r="J21" s="97" t="n"/>
-      <c r="K21" s="97" t="n"/>
-      <c r="L21" s="97" t="n"/>
-      <c r="M21" s="97" t="n"/>
-      <c r="N21" s="97" t="n"/>
-      <c r="O21" s="97" t="n"/>
-      <c r="P21" s="97" t="n"/>
-      <c r="Q21" s="97" t="n"/>
-      <c r="R21" s="97" t="n"/>
-      <c r="S21" s="97" t="n"/>
-      <c r="T21" s="97" t="n"/>
-      <c r="U21" s="97" t="n"/>
-      <c r="V21" s="97" t="n"/>
-      <c r="W21" s="97" t="n"/>
-      <c r="X21" s="97" t="n"/>
-      <c r="Y21" s="97" t="n"/>
+      <c r="A21" s="99" t="inlineStr">
+        <is>
+          <t>Chức vụ giảng viên biên soạn</t>
+        </is>
+      </c>
+      <c r="B21" s="100" t="inlineStr">
+        <is>
+          <t>TRƯỞNG BỘ MÔN</t>
+        </is>
+      </c>
+      <c r="C21" s="100" t="inlineStr">
+        <is>
+          <t>TRƯỞNG BỘ MÔN</t>
+        </is>
+      </c>
+      <c r="D21" s="100" t="n"/>
+      <c r="E21" s="100" t="n"/>
+      <c r="F21" s="100" t="n"/>
+      <c r="G21" s="100" t="n"/>
+      <c r="H21" s="100" t="n"/>
+      <c r="I21" s="100" t="n"/>
+      <c r="J21" s="100" t="n"/>
+      <c r="K21" s="100" t="n"/>
+      <c r="L21" s="100" t="n"/>
+      <c r="M21" s="100" t="n"/>
+      <c r="N21" s="100" t="n"/>
+      <c r="O21" s="100" t="n"/>
+      <c r="P21" s="100" t="n"/>
+      <c r="Q21" s="100" t="n"/>
+      <c r="R21" s="100" t="n"/>
+      <c r="S21" s="100" t="n"/>
+      <c r="T21" s="100" t="n"/>
+      <c r="U21" s="100" t="n"/>
+      <c r="V21" s="100" t="n"/>
+      <c r="W21" s="100" t="n"/>
+      <c r="X21" s="100" t="n"/>
+      <c r="Y21" s="100" t="n"/>
     </row>
     <row r="22" thickBot="1">
-      <c r="A22" s="96" t="inlineStr">
-        <is>
-          <t>Ngày thông qua</t>
-        </is>
-      </c>
-      <c r="B22" s="98" t="n">
-        <v>46118</v>
-      </c>
-      <c r="C22" s="98" t="n">
-        <v>46118</v>
-      </c>
-      <c r="D22" s="97" t="n"/>
-      <c r="E22" s="97" t="n"/>
-      <c r="F22" s="97" t="n"/>
-      <c r="G22" s="97" t="n"/>
-      <c r="H22" s="97" t="n"/>
-      <c r="I22" s="97" t="n"/>
-      <c r="J22" s="97" t="n"/>
-      <c r="K22" s="97" t="n"/>
-      <c r="L22" s="97" t="n"/>
-      <c r="M22" s="97" t="n"/>
-      <c r="N22" s="97" t="n"/>
-      <c r="O22" s="97" t="n"/>
-      <c r="P22" s="97" t="n"/>
-      <c r="Q22" s="97" t="n"/>
-      <c r="R22" s="97" t="n"/>
-      <c r="S22" s="97" t="n"/>
-      <c r="T22" s="97" t="n"/>
-      <c r="U22" s="97" t="n"/>
-      <c r="V22" s="97" t="n"/>
-      <c r="W22" s="97" t="n"/>
-      <c r="X22" s="97" t="n"/>
-      <c r="Y22" s="97" t="n"/>
+      <c r="A22" s="99" t="inlineStr">
+        <is>
+          <t>Cấp bậc, học vị, họ tên giảng viên biên soạn</t>
+        </is>
+      </c>
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>Trung tá, ThS Nguyễn Mạnh Hùng</t>
+        </is>
+      </c>
+      <c r="C22" s="100" t="inlineStr">
+        <is>
+          <t>Trung tá, ThS Nguyễn Mạnh Hùng</t>
+        </is>
+      </c>
+      <c r="D22" s="100" t="n"/>
+      <c r="E22" s="100" t="n"/>
+      <c r="F22" s="100" t="n"/>
+      <c r="G22" s="100" t="n"/>
+      <c r="H22" s="100" t="n"/>
+      <c r="I22" s="100" t="n"/>
+      <c r="J22" s="100" t="n"/>
+      <c r="K22" s="100" t="n"/>
+      <c r="L22" s="100" t="n"/>
+      <c r="M22" s="100" t="n"/>
+      <c r="N22" s="100" t="n"/>
+      <c r="O22" s="100" t="n"/>
+      <c r="P22" s="100" t="n"/>
+      <c r="Q22" s="100" t="n"/>
+      <c r="R22" s="100" t="n"/>
+      <c r="S22" s="100" t="n"/>
+      <c r="T22" s="100" t="n"/>
+      <c r="U22" s="100" t="n"/>
+      <c r="V22" s="100" t="n"/>
+      <c r="W22" s="100" t="n"/>
+      <c r="X22" s="100" t="n"/>
+      <c r="Y22" s="100" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="99" t="inlineStr">
         <is>
-          <t>Chức vụ giảng viên biên soạn</t>
-        </is>
-      </c>
-      <c r="B23" s="100" t="inlineStr">
-        <is>
-          <t>TRƯỞNG BỘ MÔN</t>
-        </is>
-      </c>
-      <c r="C23" s="100" t="inlineStr">
-        <is>
-          <t>TRƯỞNG BỘ MÔN</t>
-        </is>
+          <t>Ngày biên soạn</t>
+        </is>
+      </c>
+      <c r="B23" s="101" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C23" s="101" t="n">
+        <v>46118</v>
       </c>
       <c r="D23" s="100" t="n"/>
       <c r="E23" s="100" t="n"/>
@@ -2227,132 +2223,138 @@
       <c r="Y23" s="100" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="99" t="inlineStr">
-        <is>
-          <t>Cấp bậc, học vị giảng viên biên soạn</t>
-        </is>
-      </c>
-      <c r="B24" s="100" t="inlineStr">
-        <is>
-          <t>Trung tá, ThS</t>
-        </is>
-      </c>
-      <c r="C24" s="100" t="inlineStr">
-        <is>
-          <t>Trung tá, ThS</t>
-        </is>
-      </c>
-      <c r="D24" s="100" t="n"/>
-      <c r="E24" s="100" t="n"/>
-      <c r="F24" s="100" t="n"/>
-      <c r="G24" s="100" t="n"/>
-      <c r="H24" s="100" t="n"/>
-      <c r="I24" s="100" t="n"/>
-      <c r="J24" s="100" t="n"/>
-      <c r="K24" s="100" t="n"/>
-      <c r="L24" s="100" t="n"/>
-      <c r="M24" s="100" t="n"/>
-      <c r="N24" s="100" t="n"/>
-      <c r="O24" s="100" t="n"/>
-      <c r="P24" s="100" t="n"/>
-      <c r="Q24" s="100" t="n"/>
-      <c r="R24" s="100" t="n"/>
-      <c r="S24" s="100" t="n"/>
-      <c r="T24" s="100" t="n"/>
-      <c r="U24" s="100" t="n"/>
-      <c r="V24" s="100" t="n"/>
-      <c r="W24" s="100" t="n"/>
-      <c r="X24" s="100" t="n"/>
-      <c r="Y24" s="100" t="n"/>
+      <c r="A24" s="102" t="inlineStr">
+        <is>
+          <t>Mục đích</t>
+        </is>
+      </c>
+      <c r="B24" s="103" t="inlineStr">
+        <is>
+          <t>Sau khi học xong bài học này, học viên có khả năng phân tích công dụng, tính năng, cấu tạo chi tiết và giải thích được nguyên lý chuyển động của súng STV 380 ở các chế độ bắn, đồng thời nhận diện được các bộ phận của súng, phân biệt được các phiên bản súng tiểu liên STV dựa trên đặc điểm cấu tạo; luôn tự giác chấp hành nghiêm chỉnh quy định bảo đảm an toàn khi tiếp xúc với vũ khí.</t>
+        </is>
+      </c>
+      <c r="C24" s="103" t="inlineStr">
+        <is>
+          <t>Sau khi học xong bài học này, học viên có khả năng phân tích công dụng, tính năng, cấu tạo chi tiết và giải thích được nguyên lý chuyển động của súng STV 380 ở các chế độ bắn, đồng thời nhận diện được các bộ phận của súng, phân biệt được các phiên bản súng tiểu liên STV dựa trên đặc điểm cấu tạo; luôn tự giác chấp hành nghiêm chỉnh quy định bảo đảm an toàn khi tiếp xúc với vũ khí.</t>
+        </is>
+      </c>
+      <c r="D24" s="103" t="n"/>
+      <c r="E24" s="103" t="n"/>
+      <c r="F24" s="103" t="n"/>
+      <c r="G24" s="103" t="n"/>
+      <c r="H24" s="103" t="n"/>
+      <c r="I24" s="103" t="n"/>
+      <c r="J24" s="103" t="n"/>
+      <c r="K24" s="103" t="n"/>
+      <c r="L24" s="103" t="n"/>
+      <c r="M24" s="103" t="n"/>
+      <c r="N24" s="103" t="n"/>
+      <c r="O24" s="103" t="n"/>
+      <c r="P24" s="103" t="n"/>
+      <c r="Q24" s="103" t="n"/>
+      <c r="R24" s="103" t="n"/>
+      <c r="S24" s="103" t="n"/>
+      <c r="T24" s="103" t="n"/>
+      <c r="U24" s="103" t="n"/>
+      <c r="V24" s="103" t="n"/>
+      <c r="W24" s="103" t="n"/>
+      <c r="X24" s="103" t="n"/>
+      <c r="Y24" s="103" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="99" t="inlineStr">
-        <is>
-          <t>Họ tên giảng viên biên soạn</t>
-        </is>
-      </c>
-      <c r="B25" s="100" t="inlineStr">
-        <is>
-          <t>Nguyễn Mạnh Hùng</t>
-        </is>
-      </c>
-      <c r="C25" s="100" t="inlineStr">
-        <is>
-          <t>Nguyễn Mạnh Hùng</t>
-        </is>
-      </c>
-      <c r="D25" s="100" t="n"/>
-      <c r="E25" s="100" t="n"/>
-      <c r="F25" s="100" t="n"/>
-      <c r="G25" s="100" t="n"/>
-      <c r="H25" s="100" t="n"/>
-      <c r="I25" s="100" t="n"/>
-      <c r="J25" s="100" t="n"/>
-      <c r="K25" s="100" t="n"/>
-      <c r="L25" s="100" t="n"/>
-      <c r="M25" s="100" t="n"/>
-      <c r="N25" s="100" t="n"/>
-      <c r="O25" s="100" t="n"/>
-      <c r="P25" s="100" t="n"/>
-      <c r="Q25" s="100" t="n"/>
-      <c r="R25" s="100" t="n"/>
-      <c r="S25" s="100" t="n"/>
-      <c r="T25" s="100" t="n"/>
-      <c r="U25" s="100" t="n"/>
-      <c r="V25" s="100" t="n"/>
-      <c r="W25" s="100" t="n"/>
-      <c r="X25" s="100" t="n"/>
-      <c r="Y25" s="100" t="n"/>
+      <c r="A25" s="102" t="inlineStr">
+        <is>
+          <t>Yêu cầu về kiến thức</t>
+        </is>
+      </c>
+      <c r="B25" s="103" t="inlineStr">
+        <is>
+          <t>- Phân tích được tác dụng và cấu tạo chi tiết của các bộ phận, chi tiết chính của súng;
+- Giải thích được chuyển động của các bộ phận súng khi bắn phát một và bắn liên thanh.</t>
+        </is>
+      </c>
+      <c r="C25" s="103" t="inlineStr">
+        <is>
+          <t>- Phân tích được tác dụng và cấu tạo chi tiết của các bộ phận, chi tiết chính của súng;
+- Giải thích được chuyển động của các bộ phận súng khi bắn phát một và bắn liên thanh.</t>
+        </is>
+      </c>
+      <c r="D25" s="103" t="n"/>
+      <c r="E25" s="103" t="n"/>
+      <c r="F25" s="103" t="n"/>
+      <c r="G25" s="103" t="n"/>
+      <c r="H25" s="103" t="n"/>
+      <c r="I25" s="103" t="n"/>
+      <c r="J25" s="103" t="n"/>
+      <c r="K25" s="103" t="n"/>
+      <c r="L25" s="103" t="n"/>
+      <c r="M25" s="103" t="n"/>
+      <c r="N25" s="103" t="n"/>
+      <c r="O25" s="103" t="n"/>
+      <c r="P25" s="103" t="n"/>
+      <c r="Q25" s="103" t="n"/>
+      <c r="R25" s="103" t="n"/>
+      <c r="S25" s="103" t="n"/>
+      <c r="T25" s="103" t="n"/>
+      <c r="U25" s="103" t="n"/>
+      <c r="V25" s="103" t="n"/>
+      <c r="W25" s="103" t="n"/>
+      <c r="X25" s="103" t="n"/>
+      <c r="Y25" s="103" t="n"/>
     </row>
     <row r="26" thickBot="1">
-      <c r="A26" s="99" t="inlineStr">
-        <is>
-          <t>Ngày biên soạn</t>
-        </is>
-      </c>
-      <c r="B26" s="101" t="n">
-        <v>46118</v>
-      </c>
-      <c r="C26" s="101" t="n">
-        <v>46118</v>
-      </c>
-      <c r="D26" s="100" t="n"/>
-      <c r="E26" s="100" t="n"/>
-      <c r="F26" s="100" t="n"/>
-      <c r="G26" s="100" t="n"/>
-      <c r="H26" s="100" t="n"/>
-      <c r="I26" s="100" t="n"/>
-      <c r="J26" s="100" t="n"/>
-      <c r="K26" s="100" t="n"/>
-      <c r="L26" s="100" t="n"/>
-      <c r="M26" s="100" t="n"/>
-      <c r="N26" s="100" t="n"/>
-      <c r="O26" s="100" t="n"/>
-      <c r="P26" s="100" t="n"/>
-      <c r="Q26" s="100" t="n"/>
-      <c r="R26" s="100" t="n"/>
-      <c r="S26" s="100" t="n"/>
-      <c r="T26" s="100" t="n"/>
-      <c r="U26" s="100" t="n"/>
-      <c r="V26" s="100" t="n"/>
-      <c r="W26" s="100" t="n"/>
-      <c r="X26" s="100" t="n"/>
-      <c r="Y26" s="100" t="n"/>
+      <c r="A26" s="102" t="inlineStr">
+        <is>
+          <t>Yêu cầu về kỹ năng</t>
+        </is>
+      </c>
+      <c r="B26" s="103" t="inlineStr">
+        <is>
+          <t>Phân biệt được súng tiểu liên STV 380, STV 215 và STV 022 dựa trên các đặc điểm cấu tạo.</t>
+        </is>
+      </c>
+      <c r="C26" s="103" t="inlineStr">
+        <is>
+          <t>Phân biệt được súng tiểu liên STV 380, STV 215 và STV 022 dựa trên các đặc điểm cấu tạo.</t>
+        </is>
+      </c>
+      <c r="D26" s="103" t="n"/>
+      <c r="E26" s="103" t="n"/>
+      <c r="F26" s="103" t="n"/>
+      <c r="G26" s="103" t="n"/>
+      <c r="H26" s="103" t="n"/>
+      <c r="I26" s="103" t="n"/>
+      <c r="J26" s="103" t="n"/>
+      <c r="K26" s="103" t="n"/>
+      <c r="L26" s="103" t="n"/>
+      <c r="M26" s="103" t="n"/>
+      <c r="N26" s="103" t="n"/>
+      <c r="O26" s="103" t="n"/>
+      <c r="P26" s="103" t="n"/>
+      <c r="Q26" s="103" t="n"/>
+      <c r="R26" s="103" t="n"/>
+      <c r="S26" s="103" t="n"/>
+      <c r="T26" s="103" t="n"/>
+      <c r="U26" s="103" t="n"/>
+      <c r="V26" s="103" t="n"/>
+      <c r="W26" s="103" t="n"/>
+      <c r="X26" s="103" t="n"/>
+      <c r="Y26" s="103" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="102" t="inlineStr">
         <is>
-          <t>Mục đích</t>
+          <t>Mức tự chủ và trách nhiệm</t>
         </is>
       </c>
       <c r="B27" s="103" t="inlineStr">
         <is>
-          <t>Sau khi học xong bài học này, học viên có khả năng phân tích công dụng, tính năng, cấu tạo chi tiết và giải thích được nguyên lý chuyển động của súng STV 380 ở các chế độ bắn, đồng thời nhận diện được các bộ phận của súng, phân biệt được các phiên bản súng tiểu liên STV dựa trên đặc điểm cấu tạo; luôn tự giác chấp hành nghiêm chỉnh quy định bảo đảm an toàn khi tiếp xúc với vũ khí.</t>
+          <t>Tự giác chấp hành nghiêm các quy định an toàn khi tiếp xúc vũ khí.</t>
         </is>
       </c>
       <c r="C27" s="103" t="inlineStr">
         <is>
-          <t>Sau khi học xong bài học này, học viên có khả năng phân tích công dụng, tính năng, cấu tạo chi tiết và giải thích được nguyên lý chuyển động của súng STV 380 ở các chế độ bắn, đồng thời nhận diện được các bộ phận của súng, phân biệt được các phiên bản súng tiểu liên STV dựa trên đặc điểm cấu tạo; luôn tự giác chấp hành nghiêm chỉnh quy định bảo đảm an toàn khi tiếp xúc với vũ khí.</t>
+          <t>Tự giác chấp hành nghiêm các quy định an toàn khi tiếp xúc vũ khí.</t>
         </is>
       </c>
       <c r="D27" s="103" t="n"/>
@@ -2379,140 +2381,140 @@
       <c r="Y27" s="103" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="102" t="inlineStr">
-        <is>
-          <t>Yêu cầu về kiến thức</t>
-        </is>
-      </c>
-      <c r="B28" s="103" t="inlineStr">
-        <is>
-          <t>- Phân tích được tác dụng và cấu tạo chi tiết của các bộ phận, chi tiết chính của súng;
-- Giải thích được chuyển động của các bộ phận súng khi bắn phát một và bắn liên thanh.</t>
-        </is>
-      </c>
-      <c r="C28" s="103" t="inlineStr">
-        <is>
-          <t>- Phân tích được tác dụng và cấu tạo chi tiết của các bộ phận, chi tiết chính của súng;
-- Giải thích được chuyển động của các bộ phận súng khi bắn phát một và bắn liên thanh.</t>
-        </is>
-      </c>
-      <c r="D28" s="103" t="n"/>
-      <c r="E28" s="103" t="n"/>
-      <c r="F28" s="103" t="n"/>
-      <c r="G28" s="103" t="n"/>
-      <c r="H28" s="103" t="n"/>
-      <c r="I28" s="103" t="n"/>
-      <c r="J28" s="103" t="n"/>
-      <c r="K28" s="103" t="n"/>
-      <c r="L28" s="103" t="n"/>
-      <c r="M28" s="103" t="n"/>
-      <c r="N28" s="103" t="n"/>
-      <c r="O28" s="103" t="n"/>
-      <c r="P28" s="103" t="n"/>
-      <c r="Q28" s="103" t="n"/>
-      <c r="R28" s="103" t="n"/>
-      <c r="S28" s="103" t="n"/>
-      <c r="T28" s="103" t="n"/>
-      <c r="U28" s="103" t="n"/>
-      <c r="V28" s="103" t="n"/>
-      <c r="W28" s="103" t="n"/>
-      <c r="X28" s="103" t="n"/>
-      <c r="Y28" s="103" t="n"/>
+      <c r="A28" s="104" t="inlineStr">
+        <is>
+          <t>Nội dung bài giảng</t>
+        </is>
+      </c>
+      <c r="B28" s="105" t="inlineStr">
+        <is>
+          <t>- Cấu tạo của súng;
+- Hoạt động của súng.</t>
+        </is>
+      </c>
+      <c r="C28" s="105" t="inlineStr">
+        <is>
+          <t>- Cấu tạo của súng;
+- Hoạt động của súng.</t>
+        </is>
+      </c>
+      <c r="D28" s="105" t="n"/>
+      <c r="E28" s="105" t="n"/>
+      <c r="F28" s="105" t="n"/>
+      <c r="G28" s="105" t="n"/>
+      <c r="H28" s="105" t="n"/>
+      <c r="I28" s="105" t="n"/>
+      <c r="J28" s="105" t="n"/>
+      <c r="K28" s="105" t="n"/>
+      <c r="L28" s="105" t="n"/>
+      <c r="M28" s="105" t="n"/>
+      <c r="N28" s="105" t="n"/>
+      <c r="O28" s="105" t="n"/>
+      <c r="P28" s="105" t="n"/>
+      <c r="Q28" s="105" t="n"/>
+      <c r="R28" s="105" t="n"/>
+      <c r="S28" s="105" t="n"/>
+      <c r="T28" s="105" t="n"/>
+      <c r="U28" s="105" t="n"/>
+      <c r="V28" s="105" t="n"/>
+      <c r="W28" s="105" t="n"/>
+      <c r="X28" s="105" t="n"/>
+      <c r="Y28" s="105" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="102" t="inlineStr">
-        <is>
-          <t>Yêu cầu về kỹ năng</t>
-        </is>
-      </c>
-      <c r="B29" s="103" t="inlineStr">
-        <is>
-          <t>Phân biệt được súng tiểu liên STV 380, STV 215 và STV 022 dựa trên các đặc điểm cấu tạo.</t>
-        </is>
-      </c>
-      <c r="C29" s="103" t="inlineStr">
-        <is>
-          <t>Phân biệt được súng tiểu liên STV 380, STV 215 và STV 022 dựa trên các đặc điểm cấu tạo.</t>
-        </is>
-      </c>
-      <c r="D29" s="103" t="n"/>
-      <c r="E29" s="103" t="n"/>
-      <c r="F29" s="103" t="n"/>
-      <c r="G29" s="103" t="n"/>
-      <c r="H29" s="103" t="n"/>
-      <c r="I29" s="103" t="n"/>
-      <c r="J29" s="103" t="n"/>
-      <c r="K29" s="103" t="n"/>
-      <c r="L29" s="103" t="n"/>
-      <c r="M29" s="103" t="n"/>
-      <c r="N29" s="103" t="n"/>
-      <c r="O29" s="103" t="n"/>
-      <c r="P29" s="103" t="n"/>
-      <c r="Q29" s="103" t="n"/>
-      <c r="R29" s="103" t="n"/>
-      <c r="S29" s="103" t="n"/>
-      <c r="T29" s="103" t="n"/>
-      <c r="U29" s="103" t="n"/>
-      <c r="V29" s="103" t="n"/>
-      <c r="W29" s="103" t="n"/>
-      <c r="X29" s="103" t="n"/>
-      <c r="Y29" s="103" t="n"/>
+      <c r="A29" s="104" t="inlineStr">
+        <is>
+          <t>Tổng số thời gian</t>
+        </is>
+      </c>
+      <c r="B29" s="105" t="inlineStr">
+        <is>
+          <t>02 tiết, ngày 02 tiết; đêm 0 tiết;</t>
+        </is>
+      </c>
+      <c r="C29" s="105" t="inlineStr">
+        <is>
+          <t>02 tiết, ngày 02 tiết; đêm 0 tiết;</t>
+        </is>
+      </c>
+      <c r="D29" s="105" t="n"/>
+      <c r="E29" s="105" t="n"/>
+      <c r="F29" s="105" t="n"/>
+      <c r="G29" s="105" t="n"/>
+      <c r="H29" s="105" t="n"/>
+      <c r="I29" s="105" t="n"/>
+      <c r="J29" s="105" t="n"/>
+      <c r="K29" s="105" t="n"/>
+      <c r="L29" s="105" t="n"/>
+      <c r="M29" s="105" t="n"/>
+      <c r="N29" s="105" t="n"/>
+      <c r="O29" s="105" t="n"/>
+      <c r="P29" s="105" t="n"/>
+      <c r="Q29" s="105" t="n"/>
+      <c r="R29" s="105" t="n"/>
+      <c r="S29" s="105" t="n"/>
+      <c r="T29" s="105" t="n"/>
+      <c r="U29" s="105" t="n"/>
+      <c r="V29" s="105" t="n"/>
+      <c r="W29" s="105" t="n"/>
+      <c r="X29" s="105" t="n"/>
+      <c r="Y29" s="105" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="102" t="inlineStr">
-        <is>
-          <t>Mức tự chủ và trách nhiệm</t>
-        </is>
-      </c>
-      <c r="B30" s="103" t="inlineStr">
-        <is>
-          <t>Tự giác chấp hành nghiêm các quy định an toàn khi tiếp xúc vũ khí.</t>
-        </is>
-      </c>
-      <c r="C30" s="103" t="inlineStr">
-        <is>
-          <t>Tự giác chấp hành nghiêm các quy định an toàn khi tiếp xúc vũ khí.</t>
-        </is>
-      </c>
-      <c r="D30" s="103" t="n"/>
-      <c r="E30" s="103" t="n"/>
-      <c r="F30" s="103" t="n"/>
-      <c r="G30" s="103" t="n"/>
-      <c r="H30" s="103" t="n"/>
-      <c r="I30" s="103" t="n"/>
-      <c r="J30" s="103" t="n"/>
-      <c r="K30" s="103" t="n"/>
-      <c r="L30" s="103" t="n"/>
-      <c r="M30" s="103" t="n"/>
-      <c r="N30" s="103" t="n"/>
-      <c r="O30" s="103" t="n"/>
-      <c r="P30" s="103" t="n"/>
-      <c r="Q30" s="103" t="n"/>
-      <c r="R30" s="103" t="n"/>
-      <c r="S30" s="103" t="n"/>
-      <c r="T30" s="103" t="n"/>
-      <c r="U30" s="103" t="n"/>
-      <c r="V30" s="103" t="n"/>
-      <c r="W30" s="103" t="n"/>
-      <c r="X30" s="103" t="n"/>
-      <c r="Y30" s="103" t="n"/>
+      <c r="A30" s="104" t="inlineStr">
+        <is>
+          <t>Phân bổ thời gian</t>
+        </is>
+      </c>
+      <c r="B30" s="105" t="inlineStr">
+        <is>
+          <t>Lý thuyết: 01 tiết.
+Thảo luận: 01 tiết.</t>
+        </is>
+      </c>
+      <c r="C30" s="105" t="inlineStr">
+        <is>
+          <t>Lý thuyết: 01 tiết.
+Thảo luận: 01 tiết.</t>
+        </is>
+      </c>
+      <c r="D30" s="105" t="n"/>
+      <c r="E30" s="105" t="n"/>
+      <c r="F30" s="105" t="n"/>
+      <c r="G30" s="105" t="n"/>
+      <c r="H30" s="105" t="n"/>
+      <c r="I30" s="105" t="n"/>
+      <c r="J30" s="105" t="n"/>
+      <c r="K30" s="105" t="n"/>
+      <c r="L30" s="105" t="n"/>
+      <c r="M30" s="105" t="n"/>
+      <c r="N30" s="105" t="n"/>
+      <c r="O30" s="105" t="n"/>
+      <c r="P30" s="105" t="n"/>
+      <c r="Q30" s="105" t="n"/>
+      <c r="R30" s="105" t="n"/>
+      <c r="S30" s="105" t="n"/>
+      <c r="T30" s="105" t="n"/>
+      <c r="U30" s="105" t="n"/>
+      <c r="V30" s="105" t="n"/>
+      <c r="W30" s="105" t="n"/>
+      <c r="X30" s="105" t="n"/>
+      <c r="Y30" s="105" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="104" t="inlineStr">
         <is>
-          <t>Nội dung bài giảng</t>
+          <t>Tổ chức lớp học</t>
         </is>
       </c>
       <c r="B31" s="105" t="inlineStr">
         <is>
-          <t>- Cấu tạo của súng;
-- Hoạt động của súng.</t>
+          <t>Tổ chức theo đội hình lớp học tập trung tại phòng học lý thuyết.</t>
         </is>
       </c>
       <c r="C31" s="105" t="inlineStr">
         <is>
-          <t>- Cấu tạo của súng;
-- Hoạt động của súng.</t>
+          <t>Tổ chức theo đội hình lớp học tập trung tại phòng học lý thuyết.</t>
         </is>
       </c>
       <c r="D31" s="105" t="n"/>
@@ -2541,17 +2543,17 @@
     <row r="32">
       <c r="A32" s="104" t="inlineStr">
         <is>
-          <t>Tổng số thời gian</t>
+          <t>Phương pháp của giảng viên</t>
         </is>
       </c>
       <c r="B32" s="105" t="inlineStr">
         <is>
-          <t>02 tiết, ngày 02 tiết; đêm 0 tiết;</t>
+          <t>Thuyết trình, trao đổi, quan sát, mô phỏng.</t>
         </is>
       </c>
       <c r="C32" s="105" t="inlineStr">
         <is>
-          <t>02 tiết, ngày 02 tiết; đêm 0 tiết;</t>
+          <t>Thuyết trình, trao đổi, quan sát, mô phỏng.</t>
         </is>
       </c>
       <c r="D32" s="105" t="n"/>
@@ -2580,19 +2582,19 @@
     <row r="33">
       <c r="A33" s="104" t="inlineStr">
         <is>
-          <t>Phân bổ thời gian</t>
+          <t>Phương pháp của học viên</t>
         </is>
       </c>
       <c r="B33" s="105" t="inlineStr">
         <is>
-          <t>Lý thuyết: 01 tiết.
-Thảo luận: 01 tiết.</t>
+          <t>Giai đoạn chuẩn bị trước khi lên lớp: Tự học theo hướng dẫn trên hệ thống LMS, hoàn thành các bài kiểm tra đạt trên 80%, đặt các câu hỏi về nội dung còn thắc mắc, cần trao đổi trên diễn đàn của hệ thống LMS;
+Giai đoạn trên lớp: Nghe giảng, tương tác, thao tác, theo dõi dưới sự hướng dẫn và định hướng của giảng viên;</t>
         </is>
       </c>
       <c r="C33" s="105" t="inlineStr">
         <is>
-          <t>Lý thuyết: 01 tiết.
-Thảo luận: 01 tiết.</t>
+          <t>Giai đoạn chuẩn bị trước khi lên lớp: Tự học theo hướng dẫn trên hệ thống LMS, hoàn thành các bài kiểm tra đạt trên 80%, đặt các câu hỏi về nội dung còn thắc mắc, cần trao đổi trên diễn đàn của hệ thống LMS;
+Giai đoạn trên lớp: Nghe giảng, tương tác, thao tác, theo dõi dưới sự hướng dẫn và định hướng của giảng viên;</t>
         </is>
       </c>
       <c r="D33" s="105" t="n"/>
@@ -2621,17 +2623,17 @@
     <row r="34">
       <c r="A34" s="104" t="inlineStr">
         <is>
-          <t>Tổ chức lớp học</t>
+          <t>Phòng học</t>
         </is>
       </c>
       <c r="B34" s="105" t="inlineStr">
         <is>
-          <t>Tổ chức theo đội hình lớp học tập trung tại phòng học lý thuyết.</t>
+          <t>H2.101.</t>
         </is>
       </c>
       <c r="C34" s="105" t="inlineStr">
         <is>
-          <t>Tổ chức theo đội hình lớp học tập trung tại phòng học lý thuyết.</t>
+          <t>H2.101.</t>
         </is>
       </c>
       <c r="D34" s="105" t="n"/>
@@ -2658,131 +2660,12 @@
       <c r="Y34" s="105" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="104" t="inlineStr">
-        <is>
-          <t>Phương pháp của giảng viên</t>
-        </is>
-      </c>
-      <c r="B35" s="105" t="inlineStr">
-        <is>
-          <t>Thuyết trình, trao đổi, quan sát, mô phỏng.</t>
-        </is>
-      </c>
-      <c r="C35" s="105" t="inlineStr">
-        <is>
-          <t>Thuyết trình, trao đổi, quan sát, mô phỏng.</t>
-        </is>
-      </c>
-      <c r="D35" s="105" t="n"/>
-      <c r="E35" s="105" t="n"/>
-      <c r="F35" s="105" t="n"/>
-      <c r="G35" s="105" t="n"/>
-      <c r="H35" s="105" t="n"/>
-      <c r="I35" s="105" t="n"/>
-      <c r="J35" s="105" t="n"/>
-      <c r="K35" s="105" t="n"/>
-      <c r="L35" s="105" t="n"/>
-      <c r="M35" s="105" t="n"/>
-      <c r="N35" s="105" t="n"/>
-      <c r="O35" s="105" t="n"/>
-      <c r="P35" s="105" t="n"/>
-      <c r="Q35" s="105" t="n"/>
-      <c r="R35" s="105" t="n"/>
-      <c r="S35" s="105" t="n"/>
-      <c r="T35" s="105" t="n"/>
-      <c r="U35" s="105" t="n"/>
-      <c r="V35" s="105" t="n"/>
-      <c r="W35" s="105" t="n"/>
-      <c r="X35" s="105" t="n"/>
-      <c r="Y35" s="105" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="104" t="inlineStr">
-        <is>
-          <t>Phương pháp của học viên</t>
-        </is>
-      </c>
-      <c r="B36" s="105" t="inlineStr">
-        <is>
-          <t>Giai đoạn chuẩn bị trước khi lên lớp: Tự học theo hướng dẫn trên hệ thống LMS, hoàn thành các bài kiểm tra đạt trên 80%, đặt các câu hỏi về nội dung còn thắc mắc, cần trao đổi trên diễn đàn của hệ thống LMS;
-Giai đoạn trên lớp: Nghe giảng, tương tác, thao tác, theo dõi dưới sự hướng dẫn và định hướng của giảng viên;</t>
-        </is>
-      </c>
-      <c r="C36" s="105" t="inlineStr">
-        <is>
-          <t>Giai đoạn chuẩn bị trước khi lên lớp: Tự học theo hướng dẫn trên hệ thống LMS, hoàn thành các bài kiểm tra đạt trên 80%, đặt các câu hỏi về nội dung còn thắc mắc, cần trao đổi trên diễn đàn của hệ thống LMS;
-Giai đoạn trên lớp: Nghe giảng, tương tác, thao tác, theo dõi dưới sự hướng dẫn và định hướng của giảng viên;</t>
-        </is>
-      </c>
-      <c r="D36" s="105" t="n"/>
-      <c r="E36" s="105" t="n"/>
-      <c r="F36" s="105" t="n"/>
-      <c r="G36" s="105" t="n"/>
-      <c r="H36" s="105" t="n"/>
-      <c r="I36" s="105" t="n"/>
-      <c r="J36" s="105" t="n"/>
-      <c r="K36" s="105" t="n"/>
-      <c r="L36" s="105" t="n"/>
-      <c r="M36" s="105" t="n"/>
-      <c r="N36" s="105" t="n"/>
-      <c r="O36" s="105" t="n"/>
-      <c r="P36" s="105" t="n"/>
-      <c r="Q36" s="105" t="n"/>
-      <c r="R36" s="105" t="n"/>
-      <c r="S36" s="105" t="n"/>
-      <c r="T36" s="105" t="n"/>
-      <c r="U36" s="105" t="n"/>
-      <c r="V36" s="105" t="n"/>
-      <c r="W36" s="105" t="n"/>
-      <c r="X36" s="105" t="n"/>
-      <c r="Y36" s="105" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="104" t="inlineStr">
-        <is>
-          <t>Phòng học</t>
-        </is>
-      </c>
-      <c r="B37" s="105" t="inlineStr">
-        <is>
-          <t>H2.101.</t>
-        </is>
-      </c>
-      <c r="C37" s="105" t="inlineStr">
-        <is>
-          <t>H2.101.</t>
-        </is>
-      </c>
-      <c r="D37" s="105" t="n"/>
-      <c r="E37" s="105" t="n"/>
-      <c r="F37" s="105" t="n"/>
-      <c r="G37" s="105" t="n"/>
-      <c r="H37" s="105" t="n"/>
-      <c r="I37" s="105" t="n"/>
-      <c r="J37" s="105" t="n"/>
-      <c r="K37" s="105" t="n"/>
-      <c r="L37" s="105" t="n"/>
-      <c r="M37" s="105" t="n"/>
-      <c r="N37" s="105" t="n"/>
-      <c r="O37" s="105" t="n"/>
-      <c r="P37" s="105" t="n"/>
-      <c r="Q37" s="105" t="n"/>
-      <c r="R37" s="105" t="n"/>
-      <c r="S37" s="105" t="n"/>
-      <c r="T37" s="105" t="n"/>
-      <c r="U37" s="105" t="n"/>
-      <c r="V37" s="105" t="n"/>
-      <c r="W37" s="105" t="n"/>
-      <c r="X37" s="105" t="n"/>
-      <c r="Y37" s="105" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="106" t="inlineStr">
+      <c r="A35" s="106" t="inlineStr">
         <is>
           <t>Vật chất bảo đảm của giảng viên</t>
         </is>
       </c>
-      <c r="B38" s="107" t="inlineStr">
+      <c r="B35" s="107" t="inlineStr">
         <is>
           <t>- Kế hoạch giảng bài, bài giảng;
 - Súng tiểu liên STV 380: 03 khẩu;
@@ -2790,12 +2673,129 @@
 - Tài liệu học tập chính: Lương Văn Thuận (2023). Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật quân sự</t>
         </is>
       </c>
-      <c r="C38" s="107" t="inlineStr">
+      <c r="C35" s="107" t="inlineStr">
         <is>
           <t>- Kế hoạch giảng bài, bài giảng;
 - Súng tiểu liên STV 380: 03 khẩu;
 - Tranh cấu tạo và hoạt động: 02 tranh;
 - Tài liệu học tập chính: Lương Văn Thuận (2023). Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật quân sự</t>
+        </is>
+      </c>
+      <c r="D35" s="107" t="n"/>
+      <c r="E35" s="107" t="n"/>
+      <c r="F35" s="107" t="n"/>
+      <c r="G35" s="107" t="n"/>
+      <c r="H35" s="107" t="n"/>
+      <c r="I35" s="107" t="n"/>
+      <c r="J35" s="107" t="n"/>
+      <c r="K35" s="107" t="n"/>
+      <c r="L35" s="107" t="n"/>
+      <c r="M35" s="107" t="n"/>
+      <c r="N35" s="107" t="n"/>
+      <c r="O35" s="107" t="n"/>
+      <c r="P35" s="107" t="n"/>
+      <c r="Q35" s="107" t="n"/>
+      <c r="R35" s="107" t="n"/>
+      <c r="S35" s="107" t="n"/>
+      <c r="T35" s="107" t="n"/>
+      <c r="U35" s="107" t="n"/>
+      <c r="V35" s="107" t="n"/>
+      <c r="W35" s="107" t="n"/>
+      <c r="X35" s="107" t="n"/>
+      <c r="Y35" s="107" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="106" t="inlineStr">
+        <is>
+          <t>Vật chất bảo đảm của học viên</t>
+        </is>
+      </c>
+      <c r="B36" s="107" t="inlineStr">
+        <is>
+          <t>- Các vật chất bảo đảm việc ghi chép nội dung bài giảng;</t>
+        </is>
+      </c>
+      <c r="C36" s="107" t="inlineStr">
+        <is>
+          <t>- Các vật chất bảo đảm việc ghi chép nội dung bài giảng;</t>
+        </is>
+      </c>
+      <c r="D36" s="107" t="n"/>
+      <c r="E36" s="107" t="n"/>
+      <c r="F36" s="107" t="n"/>
+      <c r="G36" s="107" t="n"/>
+      <c r="H36" s="107" t="n"/>
+      <c r="I36" s="107" t="n"/>
+      <c r="J36" s="107" t="n"/>
+      <c r="K36" s="107" t="n"/>
+      <c r="L36" s="107" t="n"/>
+      <c r="M36" s="107" t="n"/>
+      <c r="N36" s="107" t="n"/>
+      <c r="O36" s="107" t="n"/>
+      <c r="P36" s="107" t="n"/>
+      <c r="Q36" s="107" t="n"/>
+      <c r="R36" s="107" t="n"/>
+      <c r="S36" s="107" t="n"/>
+      <c r="T36" s="107" t="n"/>
+      <c r="U36" s="107" t="n"/>
+      <c r="V36" s="107" t="n"/>
+      <c r="W36" s="107" t="n"/>
+      <c r="X36" s="107" t="n"/>
+      <c r="Y36" s="107" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="106" t="inlineStr">
+        <is>
+          <t>Tài liệu học tập chính</t>
+        </is>
+      </c>
+      <c r="B37" s="107" t="inlineStr">
+        <is>
+          <t>Lương Văn Thuận. Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật Quân sự (2023)</t>
+        </is>
+      </c>
+      <c r="C37" s="107" t="inlineStr">
+        <is>
+          <t>Lương Văn Thuận. Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật Quân sự (2023)</t>
+        </is>
+      </c>
+      <c r="D37" s="107" t="n"/>
+      <c r="E37" s="107" t="n"/>
+      <c r="F37" s="107" t="n"/>
+      <c r="G37" s="107" t="n"/>
+      <c r="H37" s="107" t="n"/>
+      <c r="I37" s="107" t="n"/>
+      <c r="J37" s="107" t="n"/>
+      <c r="K37" s="107" t="n"/>
+      <c r="L37" s="107" t="n"/>
+      <c r="M37" s="107" t="n"/>
+      <c r="N37" s="107" t="n"/>
+      <c r="O37" s="107" t="n"/>
+      <c r="P37" s="107" t="n"/>
+      <c r="Q37" s="107" t="n"/>
+      <c r="R37" s="107" t="n"/>
+      <c r="S37" s="107" t="n"/>
+      <c r="T37" s="107" t="n"/>
+      <c r="U37" s="107" t="n"/>
+      <c r="V37" s="107" t="n"/>
+      <c r="W37" s="107" t="n"/>
+      <c r="X37" s="107" t="n"/>
+      <c r="Y37" s="107" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="106" t="inlineStr">
+        <is>
+          <t>Tài liệu tham khảo</t>
+        </is>
+      </c>
+      <c r="B38" s="107" t="inlineStr">
+        <is>
+          <t>Nguyễn Mạnh Hùng, Vũ khí bộ binh, Trường Sĩ quan Kỹ thuật Quân sự (2015)</t>
+        </is>
+      </c>
+      <c r="C38" s="107" t="inlineStr">
+        <is>
+          <t>Nguyễn Mạnh Hùng, Vũ khí bộ binh, Trường Sĩ quan Kỹ thuật Quân sự (2015)</t>
         </is>
       </c>
       <c r="D38" s="107" t="n"/>
@@ -2822,133 +2822,121 @@
       <c r="Y38" s="107" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="106" t="inlineStr">
-        <is>
-          <t>Vật chất bảo đảm của học viên</t>
-        </is>
-      </c>
-      <c r="B39" s="107" t="inlineStr">
-        <is>
-          <t>- Các vật chất bảo đảm việc ghi chép nội dung bài giảng;</t>
-        </is>
-      </c>
-      <c r="C39" s="107" t="inlineStr">
-        <is>
-          <t>- Các vật chất bảo đảm việc ghi chép nội dung bài giảng;</t>
-        </is>
-      </c>
-      <c r="D39" s="107" t="n"/>
-      <c r="E39" s="107" t="n"/>
-      <c r="F39" s="107" t="n"/>
-      <c r="G39" s="107" t="n"/>
-      <c r="H39" s="107" t="n"/>
-      <c r="I39" s="107" t="n"/>
-      <c r="J39" s="107" t="n"/>
-      <c r="K39" s="107" t="n"/>
-      <c r="L39" s="107" t="n"/>
-      <c r="M39" s="107" t="n"/>
-      <c r="N39" s="107" t="n"/>
-      <c r="O39" s="107" t="n"/>
-      <c r="P39" s="107" t="n"/>
-      <c r="Q39" s="107" t="n"/>
-      <c r="R39" s="107" t="n"/>
-      <c r="S39" s="107" t="n"/>
-      <c r="T39" s="107" t="n"/>
-      <c r="U39" s="107" t="n"/>
-      <c r="V39" s="107" t="n"/>
-      <c r="W39" s="107" t="n"/>
-      <c r="X39" s="107" t="n"/>
-      <c r="Y39" s="107" t="n"/>
+      <c r="A39" s="108" t="inlineStr">
+        <is>
+          <t>Thời gian thực hành giảng bài</t>
+        </is>
+      </c>
+      <c r="B39" s="109" t="n">
+        <v>90</v>
+      </c>
+      <c r="C39" s="109" t="n">
+        <v>90</v>
+      </c>
+      <c r="D39" s="109" t="n"/>
+      <c r="E39" s="109" t="n"/>
+      <c r="F39" s="109" t="n"/>
+      <c r="G39" s="109" t="n"/>
+      <c r="H39" s="109" t="n"/>
+      <c r="I39" s="109" t="n"/>
+      <c r="J39" s="109" t="n"/>
+      <c r="K39" s="109" t="n"/>
+      <c r="L39" s="109" t="n"/>
+      <c r="M39" s="109" t="n"/>
+      <c r="N39" s="109" t="n"/>
+      <c r="O39" s="109" t="n"/>
+      <c r="P39" s="109" t="n"/>
+      <c r="Q39" s="109" t="n"/>
+      <c r="R39" s="109" t="n"/>
+      <c r="S39" s="109" t="n"/>
+      <c r="T39" s="109" t="n"/>
+      <c r="U39" s="109" t="n"/>
+      <c r="V39" s="109" t="n"/>
+      <c r="W39" s="109" t="n"/>
+      <c r="X39" s="109" t="n"/>
+      <c r="Y39" s="109" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="106" t="inlineStr">
-        <is>
-          <t>Tài liệu học tập chính</t>
-        </is>
-      </c>
-      <c r="B40" s="107" t="inlineStr">
-        <is>
-          <t>Lương Văn Thuận. Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật Quân sự (2023)</t>
-        </is>
-      </c>
-      <c r="C40" s="107" t="inlineStr">
-        <is>
-          <t>Lương Văn Thuận. Súng tiểu liên STV 215, STV 380. Trường Sĩ quan Kỹ thuật Quân sự (2023)</t>
-        </is>
-      </c>
-      <c r="D40" s="107" t="n"/>
-      <c r="E40" s="107" t="n"/>
-      <c r="F40" s="107" t="n"/>
-      <c r="G40" s="107" t="n"/>
-      <c r="H40" s="107" t="n"/>
-      <c r="I40" s="107" t="n"/>
-      <c r="J40" s="107" t="n"/>
-      <c r="K40" s="107" t="n"/>
-      <c r="L40" s="107" t="n"/>
-      <c r="M40" s="107" t="n"/>
-      <c r="N40" s="107" t="n"/>
-      <c r="O40" s="107" t="n"/>
-      <c r="P40" s="107" t="n"/>
-      <c r="Q40" s="107" t="n"/>
-      <c r="R40" s="107" t="n"/>
-      <c r="S40" s="107" t="n"/>
-      <c r="T40" s="107" t="n"/>
-      <c r="U40" s="107" t="n"/>
-      <c r="V40" s="107" t="n"/>
-      <c r="W40" s="107" t="n"/>
-      <c r="X40" s="107" t="n"/>
-      <c r="Y40" s="107" t="n"/>
+      <c r="A40" s="108" t="inlineStr">
+        <is>
+          <t>Thời gian thủ tục giảng bài</t>
+        </is>
+      </c>
+      <c r="B40" s="109" t="n">
+        <v>10</v>
+      </c>
+      <c r="C40" s="109" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="109" t="n"/>
+      <c r="E40" s="109" t="n"/>
+      <c r="F40" s="109" t="n"/>
+      <c r="G40" s="109" t="n"/>
+      <c r="H40" s="109" t="n"/>
+      <c r="I40" s="109" t="n"/>
+      <c r="J40" s="109" t="n"/>
+      <c r="K40" s="109" t="n"/>
+      <c r="L40" s="109" t="n"/>
+      <c r="M40" s="109" t="n"/>
+      <c r="N40" s="109" t="n"/>
+      <c r="O40" s="109" t="n"/>
+      <c r="P40" s="109" t="n"/>
+      <c r="Q40" s="109" t="n"/>
+      <c r="R40" s="109" t="n"/>
+      <c r="S40" s="109" t="n"/>
+      <c r="T40" s="109" t="n"/>
+      <c r="U40" s="109" t="n"/>
+      <c r="V40" s="109" t="n"/>
+      <c r="W40" s="109" t="n"/>
+      <c r="X40" s="109" t="n"/>
+      <c r="Y40" s="109" t="n"/>
     </row>
     <row r="41" thickBot="1">
-      <c r="A41" s="106" t="inlineStr">
-        <is>
-          <t>Tài liệu tham khảo</t>
-        </is>
-      </c>
-      <c r="B41" s="107" t="inlineStr">
-        <is>
-          <t>Nguyễn Mạnh Hùng, Vũ khí bộ binh, Trường Sĩ quan Kỹ thuật Quân sự (2015)</t>
-        </is>
-      </c>
-      <c r="C41" s="107" t="inlineStr">
-        <is>
-          <t>Nguyễn Mạnh Hùng, Vũ khí bộ binh, Trường Sĩ quan Kỹ thuật Quân sự (2015)</t>
-        </is>
-      </c>
-      <c r="D41" s="107" t="n"/>
-      <c r="E41" s="107" t="n"/>
-      <c r="F41" s="107" t="n"/>
-      <c r="G41" s="107" t="n"/>
-      <c r="H41" s="107" t="n"/>
-      <c r="I41" s="107" t="n"/>
-      <c r="J41" s="107" t="n"/>
-      <c r="K41" s="107" t="n"/>
-      <c r="L41" s="107" t="n"/>
-      <c r="M41" s="107" t="n"/>
-      <c r="N41" s="107" t="n"/>
-      <c r="O41" s="107" t="n"/>
-      <c r="P41" s="107" t="n"/>
-      <c r="Q41" s="107" t="n"/>
-      <c r="R41" s="107" t="n"/>
-      <c r="S41" s="107" t="n"/>
-      <c r="T41" s="107" t="n"/>
-      <c r="U41" s="107" t="n"/>
-      <c r="V41" s="107" t="n"/>
-      <c r="W41" s="107" t="n"/>
-      <c r="X41" s="107" t="n"/>
-      <c r="Y41" s="107" t="n"/>
+      <c r="A41" s="108" t="inlineStr">
+        <is>
+          <t>Thời gian nội dung bài giảng</t>
+        </is>
+      </c>
+      <c r="B41" s="109" t="n">
+        <v>75</v>
+      </c>
+      <c r="C41" s="109" t="n">
+        <v>75</v>
+      </c>
+      <c r="D41" s="109" t="n"/>
+      <c r="E41" s="109" t="n"/>
+      <c r="F41" s="109" t="n"/>
+      <c r="G41" s="109" t="n"/>
+      <c r="H41" s="109" t="n"/>
+      <c r="I41" s="109" t="n"/>
+      <c r="J41" s="109" t="n"/>
+      <c r="K41" s="109" t="n"/>
+      <c r="L41" s="109" t="n"/>
+      <c r="M41" s="109" t="n"/>
+      <c r="N41" s="109" t="n"/>
+      <c r="O41" s="109" t="n"/>
+      <c r="P41" s="109" t="n"/>
+      <c r="Q41" s="109" t="n"/>
+      <c r="R41" s="109" t="n"/>
+      <c r="S41" s="109" t="n"/>
+      <c r="T41" s="109" t="n"/>
+      <c r="U41" s="109" t="n"/>
+      <c r="V41" s="109" t="n"/>
+      <c r="W41" s="109" t="n"/>
+      <c r="X41" s="109" t="n"/>
+      <c r="Y41" s="109" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="108" t="inlineStr">
         <is>
-          <t>Thời gian thực hành giảng bài</t>
+          <t>Thời gian mở đầu</t>
         </is>
       </c>
       <c r="B42" s="109" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="C42" s="109" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="D42" s="109" t="n"/>
       <c r="E42" s="109" t="n"/>
@@ -2976,14 +2964,14 @@
     <row r="43">
       <c r="A43" s="108" t="inlineStr">
         <is>
-          <t>Thời gian thủ tục giảng bài</t>
+          <t>Thời gian phần nội dung</t>
         </is>
       </c>
       <c r="B43" s="109" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C43" s="109" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="D43" s="109" t="n"/>
       <c r="E43" s="109" t="n"/>
@@ -3011,14 +2999,14 @@
     <row r="44">
       <c r="A44" s="108" t="inlineStr">
         <is>
-          <t>Thời gian nội dung bài giảng</t>
+          <t>Thời gian kết luận</t>
         </is>
       </c>
       <c r="B44" s="109" t="n">
-        <v>75</v>
+        <v>5</v>
       </c>
       <c r="C44" s="109" t="n">
-        <v>75</v>
+        <v>5</v>
       </c>
       <c r="D44" s="109" t="n"/>
       <c r="E44" s="109" t="n"/>
@@ -3046,7 +3034,7 @@
     <row r="45">
       <c r="A45" s="108" t="inlineStr">
         <is>
-          <t>Thời gian mở đầu</t>
+          <t>Thời gian kết thúc giảng bài</t>
         </is>
       </c>
       <c r="B45" s="109" t="n">
@@ -3079,199 +3067,94 @@
       <c r="Y45" s="109" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="108" t="inlineStr">
-        <is>
-          <t>Thời gian phần nội dung</t>
-        </is>
-      </c>
-      <c r="B46" s="109" t="n">
-        <v>70</v>
-      </c>
-      <c r="C46" s="109" t="n">
-        <v>70</v>
-      </c>
-      <c r="D46" s="109" t="n"/>
-      <c r="E46" s="109" t="n"/>
-      <c r="F46" s="109" t="n"/>
-      <c r="G46" s="109" t="n"/>
-      <c r="H46" s="109" t="n"/>
-      <c r="I46" s="109" t="n"/>
-      <c r="J46" s="109" t="n"/>
-      <c r="K46" s="109" t="n"/>
-      <c r="L46" s="109" t="n"/>
-      <c r="M46" s="109" t="n"/>
-      <c r="N46" s="109" t="n"/>
-      <c r="O46" s="109" t="n"/>
-      <c r="P46" s="109" t="n"/>
-      <c r="Q46" s="109" t="n"/>
-      <c r="R46" s="109" t="n"/>
-      <c r="S46" s="109" t="n"/>
-      <c r="T46" s="109" t="n"/>
-      <c r="U46" s="109" t="n"/>
-      <c r="V46" s="109" t="n"/>
-      <c r="W46" s="109" t="n"/>
-      <c r="X46" s="109" t="n"/>
-      <c r="Y46" s="109" t="n"/>
-    </row>
-    <row r="47" thickBot="1">
-      <c r="A47" s="108" t="inlineStr">
-        <is>
-          <t>Thời gian kết luận</t>
-        </is>
-      </c>
-      <c r="B47" s="109" t="n">
-        <v>5</v>
-      </c>
-      <c r="C47" s="109" t="n">
-        <v>5</v>
-      </c>
-      <c r="D47" s="109" t="n"/>
-      <c r="E47" s="109" t="n"/>
-      <c r="F47" s="109" t="n"/>
-      <c r="G47" s="109" t="n"/>
-      <c r="H47" s="109" t="n"/>
-      <c r="I47" s="109" t="n"/>
-      <c r="J47" s="109" t="n"/>
-      <c r="K47" s="109" t="n"/>
-      <c r="L47" s="109" t="n"/>
-      <c r="M47" s="109" t="n"/>
-      <c r="N47" s="109" t="n"/>
-      <c r="O47" s="109" t="n"/>
-      <c r="P47" s="109" t="n"/>
-      <c r="Q47" s="109" t="n"/>
-      <c r="R47" s="109" t="n"/>
-      <c r="S47" s="109" t="n"/>
-      <c r="T47" s="109" t="n"/>
-      <c r="U47" s="109" t="n"/>
-      <c r="V47" s="109" t="n"/>
-      <c r="W47" s="109" t="n"/>
-      <c r="X47" s="109" t="n"/>
-      <c r="Y47" s="109" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="108" t="inlineStr">
-        <is>
-          <t>Thời gian kết thúc giảng bài</t>
-        </is>
-      </c>
-      <c r="B48" s="109" t="n">
-        <v>5</v>
-      </c>
-      <c r="C48" s="109" t="n">
-        <v>5</v>
-      </c>
-      <c r="D48" s="109" t="n"/>
-      <c r="E48" s="109" t="n"/>
-      <c r="F48" s="109" t="n"/>
-      <c r="G48" s="109" t="n"/>
-      <c r="H48" s="109" t="n"/>
-      <c r="I48" s="109" t="n"/>
-      <c r="J48" s="109" t="n"/>
-      <c r="K48" s="109" t="n"/>
-      <c r="L48" s="109" t="n"/>
-      <c r="M48" s="109" t="n"/>
-      <c r="N48" s="109" t="n"/>
-      <c r="O48" s="109" t="n"/>
-      <c r="P48" s="109" t="n"/>
-      <c r="Q48" s="109" t="n"/>
-      <c r="R48" s="109" t="n"/>
-      <c r="S48" s="109" t="n"/>
-      <c r="T48" s="109" t="n"/>
-      <c r="U48" s="109" t="n"/>
-      <c r="V48" s="109" t="n"/>
-      <c r="W48" s="109" t="n"/>
-      <c r="X48" s="109" t="n"/>
-      <c r="Y48" s="109" t="n"/>
-    </row>
-    <row r="49" thickBot="1">
-      <c r="A49" s="110" t="inlineStr">
+      <c r="A46" s="110" t="inlineStr">
         <is>
           <t>Nội dung mở đầu bài giảng</t>
         </is>
       </c>
-      <c r="B49" s="111" t="inlineStr">
+      <c r="B46" s="111" t="inlineStr">
         <is>
           <t>- Ổn định lớp, kiểm tra quân số, trang phục, vật chất học tập;
 - Quán triệt mục đích, yêu cầu và nội dung buổi học.</t>
         </is>
       </c>
-      <c r="C49" s="111" t="inlineStr">
+      <c r="C46" s="111" t="inlineStr">
         <is>
           <t>- Ổn định lớp, kiểm tra quân số, trang phục, vật chất học tập;
 - Quán triệt mục đích, yêu cầu và nội dung buổi học.</t>
         </is>
       </c>
-      <c r="D49" s="111" t="n"/>
-      <c r="E49" s="111" t="n"/>
-      <c r="F49" s="111" t="n"/>
-      <c r="G49" s="111" t="n"/>
-      <c r="H49" s="111" t="n"/>
-      <c r="I49" s="111" t="n"/>
-      <c r="J49" s="111" t="n"/>
-      <c r="K49" s="111" t="n"/>
-      <c r="L49" s="111" t="n"/>
-      <c r="M49" s="111" t="n"/>
-      <c r="N49" s="111" t="n"/>
-      <c r="O49" s="111" t="n"/>
-      <c r="P49" s="111" t="n"/>
-      <c r="Q49" s="111" t="n"/>
-      <c r="R49" s="111" t="n"/>
-      <c r="S49" s="111" t="n"/>
-      <c r="T49" s="111" t="n"/>
-      <c r="U49" s="111" t="n"/>
-      <c r="V49" s="111" t="n"/>
-      <c r="W49" s="111" t="n"/>
-      <c r="X49" s="111" t="n"/>
-      <c r="Y49" s="111" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="110" t="inlineStr">
+      <c r="D46" s="111" t="n"/>
+      <c r="E46" s="111" t="n"/>
+      <c r="F46" s="111" t="n"/>
+      <c r="G46" s="111" t="n"/>
+      <c r="H46" s="111" t="n"/>
+      <c r="I46" s="111" t="n"/>
+      <c r="J46" s="111" t="n"/>
+      <c r="K46" s="111" t="n"/>
+      <c r="L46" s="111" t="n"/>
+      <c r="M46" s="111" t="n"/>
+      <c r="N46" s="111" t="n"/>
+      <c r="O46" s="111" t="n"/>
+      <c r="P46" s="111" t="n"/>
+      <c r="Q46" s="111" t="n"/>
+      <c r="R46" s="111" t="n"/>
+      <c r="S46" s="111" t="n"/>
+      <c r="T46" s="111" t="n"/>
+      <c r="U46" s="111" t="n"/>
+      <c r="V46" s="111" t="n"/>
+      <c r="W46" s="111" t="n"/>
+      <c r="X46" s="111" t="n"/>
+      <c r="Y46" s="111" t="n"/>
+    </row>
+    <row r="47" thickBot="1">
+      <c r="A47" s="110" t="inlineStr">
         <is>
           <t>Nội dung kết luận bài giảng</t>
         </is>
       </c>
-      <c r="B50" s="111" t="inlineStr">
+      <c r="B47" s="111" t="inlineStr">
         <is>
           <t>- Tóm tắt các nội dung trọng tâm của bài học;
 - Tuyên dương các cá nhân, tổ nhóm học tập tốt.</t>
         </is>
       </c>
-      <c r="C50" s="111" t="inlineStr">
+      <c r="C47" s="111" t="inlineStr">
         <is>
           <t>- Tóm tắt các nội dung trọng tâm của bài học;
 - Tuyên dương các cá nhân, tổ nhóm học tập tốt.</t>
         </is>
       </c>
-      <c r="D50" s="111" t="n"/>
-      <c r="E50" s="111" t="n"/>
-      <c r="F50" s="111" t="n"/>
-      <c r="G50" s="111" t="n"/>
-      <c r="H50" s="111" t="n"/>
-      <c r="I50" s="111" t="n"/>
-      <c r="J50" s="111" t="n"/>
-      <c r="K50" s="111" t="n"/>
-      <c r="L50" s="111" t="n"/>
-      <c r="M50" s="111" t="n"/>
-      <c r="N50" s="111" t="n"/>
-      <c r="O50" s="111" t="n"/>
-      <c r="P50" s="111" t="n"/>
-      <c r="Q50" s="111" t="n"/>
-      <c r="R50" s="111" t="n"/>
-      <c r="S50" s="111" t="n"/>
-      <c r="T50" s="111" t="n"/>
-      <c r="U50" s="111" t="n"/>
-      <c r="V50" s="111" t="n"/>
-      <c r="W50" s="111" t="n"/>
-      <c r="X50" s="111" t="n"/>
-      <c r="Y50" s="111" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="110" t="inlineStr">
+      <c r="D47" s="111" t="n"/>
+      <c r="E47" s="111" t="n"/>
+      <c r="F47" s="111" t="n"/>
+      <c r="G47" s="111" t="n"/>
+      <c r="H47" s="111" t="n"/>
+      <c r="I47" s="111" t="n"/>
+      <c r="J47" s="111" t="n"/>
+      <c r="K47" s="111" t="n"/>
+      <c r="L47" s="111" t="n"/>
+      <c r="M47" s="111" t="n"/>
+      <c r="N47" s="111" t="n"/>
+      <c r="O47" s="111" t="n"/>
+      <c r="P47" s="111" t="n"/>
+      <c r="Q47" s="111" t="n"/>
+      <c r="R47" s="111" t="n"/>
+      <c r="S47" s="111" t="n"/>
+      <c r="T47" s="111" t="n"/>
+      <c r="U47" s="111" t="n"/>
+      <c r="V47" s="111" t="n"/>
+      <c r="W47" s="111" t="n"/>
+      <c r="X47" s="111" t="n"/>
+      <c r="Y47" s="111" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="110" t="inlineStr">
         <is>
           <t>Nội dung kết thúc giảng bài</t>
         </is>
       </c>
-      <c r="B51" s="111" t="inlineStr">
+      <c r="B48" s="111" t="inlineStr">
         <is>
           <t>- Hệ thống nội dung bài giảng;
 - Giải đáp thắc mắc;
@@ -3279,7 +3162,7 @@
 - Nhận xét, kết thúc bài giảng.</t>
         </is>
       </c>
-      <c r="C51" s="111" t="inlineStr">
+      <c r="C48" s="111" t="inlineStr">
         <is>
           <t>- Hệ thống nội dung bài giảng;
 - Giải đáp thắc mắc;
@@ -3287,207 +3170,210 @@
 - Nhận xét, kết thúc bài giảng.</t>
         </is>
       </c>
-      <c r="D51" s="111" t="n"/>
-      <c r="E51" s="111" t="n"/>
-      <c r="F51" s="111" t="n"/>
-      <c r="G51" s="111" t="n"/>
-      <c r="H51" s="111" t="n"/>
-      <c r="I51" s="111" t="n"/>
-      <c r="J51" s="111" t="n"/>
-      <c r="K51" s="111" t="n"/>
-      <c r="L51" s="111" t="n"/>
-      <c r="M51" s="111" t="n"/>
-      <c r="N51" s="111" t="n"/>
-      <c r="O51" s="111" t="n"/>
-      <c r="P51" s="111" t="n"/>
-      <c r="Q51" s="111" t="n"/>
-      <c r="R51" s="111" t="n"/>
-      <c r="S51" s="111" t="n"/>
-      <c r="T51" s="111" t="n"/>
-      <c r="U51" s="111" t="n"/>
-      <c r="V51" s="111" t="n"/>
-      <c r="W51" s="111" t="n"/>
-      <c r="X51" s="111" t="n"/>
-      <c r="Y51" s="111" t="n"/>
-    </row>
-    <row r="52" ht="45" customHeight="1"/>
+      <c r="D48" s="111" t="n"/>
+      <c r="E48" s="111" t="n"/>
+      <c r="F48" s="111" t="n"/>
+      <c r="G48" s="111" t="n"/>
+      <c r="H48" s="111" t="n"/>
+      <c r="I48" s="111" t="n"/>
+      <c r="J48" s="111" t="n"/>
+      <c r="K48" s="111" t="n"/>
+      <c r="L48" s="111" t="n"/>
+      <c r="M48" s="111" t="n"/>
+      <c r="N48" s="111" t="n"/>
+      <c r="O48" s="111" t="n"/>
+      <c r="P48" s="111" t="n"/>
+      <c r="Q48" s="111" t="n"/>
+      <c r="R48" s="111" t="n"/>
+      <c r="S48" s="111" t="n"/>
+      <c r="T48" s="111" t="n"/>
+      <c r="U48" s="111" t="n"/>
+      <c r="V48" s="111" t="n"/>
+      <c r="W48" s="111" t="n"/>
+      <c r="X48" s="111" t="n"/>
+      <c r="Y48" s="111" t="n"/>
+    </row>
+    <row r="49" thickBot="1"/>
+    <row r="50">
+      <c r="A50" s="33" t="inlineStr">
+        <is>
+          <t>HƯỚNG DẪN NHẬP LIỆU</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="34" t="inlineStr">
+        <is>
+          <t>Bố cục bảng</t>
+        </is>
+      </c>
+      <c r="B51" s="35" t="inlineStr">
+        <is>
+          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
+        </is>
+      </c>
+      <c r="C51" s="35" t="inlineStr">
+        <is>
+          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="A52" s="34" t="inlineStr">
+        <is>
+          <t>Cột A</t>
+        </is>
+      </c>
+      <c r="B52" s="35" t="inlineStr">
+        <is>
+          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
+        </is>
+      </c>
+      <c r="C52" s="35" t="inlineStr">
+        <is>
+          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
+        </is>
+      </c>
+    </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="33" t="inlineStr">
-        <is>
-          <t>HƯỚNG DẪN NHẬP LIỆU</t>
+      <c r="A53" s="34" t="inlineStr">
+        <is>
+          <t>Cột B</t>
+        </is>
+      </c>
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
+        </is>
+      </c>
+      <c r="C53" s="35" t="inlineStr">
+        <is>
+          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>Bố cục bảng</t>
+          <t>Ô nhiều dòng</t>
         </is>
       </c>
       <c r="B54" s="35" t="inlineStr">
         <is>
-          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
+          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
         </is>
       </c>
       <c r="C54" s="35" t="inlineStr">
         <is>
-          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
+          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="34" t="inlineStr">
         <is>
-          <t>Cột A</t>
+          <t>Ô ngày tháng</t>
         </is>
       </c>
       <c r="B55" s="35" t="inlineStr">
         <is>
-          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
+          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
         </is>
       </c>
       <c r="C55" s="35" t="inlineStr">
         <is>
-          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
+          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="34" t="inlineStr">
         <is>
-          <t>Cột B</t>
+          <t>Cú pháp mẫu Word</t>
         </is>
       </c>
       <c r="B56" s="35" t="inlineStr">
         <is>
-          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
+          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
         </is>
       </c>
       <c r="C56" s="35" t="inlineStr">
         <is>
-          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
+          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="34" t="inlineStr">
         <is>
-          <t>Ô nhiều dòng</t>
+          <t>Ký hiệu định dạng</t>
         </is>
       </c>
       <c r="B57" s="35" t="inlineStr">
         <is>
-          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
+          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
         </is>
       </c>
       <c r="C57" s="35" t="inlineStr">
         <is>
-          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
+          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
         <is>
-          <t>Ô ngày tháng</t>
+          <t>Trang bìa</t>
         </is>
       </c>
       <c r="B58" s="35" t="inlineStr">
         <is>
-          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
+          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
         </is>
       </c>
       <c r="C58" s="35" t="inlineStr">
         <is>
-          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
+          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="34" t="inlineStr">
         <is>
-          <t>Cú pháp mẫu Word</t>
+          <t>Trường dùng chung</t>
         </is>
       </c>
       <c r="B59" s="35" t="inlineStr">
         <is>
-          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
+          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
         </is>
       </c>
       <c r="C59" s="35" t="inlineStr">
         <is>
-          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
+          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="34" t="inlineStr">
         <is>
-          <t>Ký hiệu định dạng</t>
+          <t>Định dạng chữ</t>
         </is>
       </c>
       <c r="B60" s="35" t="inlineStr">
         <is>
-          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
+          <t>Mỗi vị trí trong Word giữ nguyên đậm / nghiêng / in hoa / căn lề của bản gốc, kể cả khi dùng chung một trường. Phần mềm chỉ thay chữ, không đụng tới định dạng.</t>
         </is>
       </c>
       <c r="C60" s="35" t="inlineStr">
         <is>
-          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="34" t="inlineStr">
-        <is>
-          <t>Trang bìa</t>
-        </is>
-      </c>
-      <c r="B61" s="35" t="inlineStr">
-        <is>
-          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
-        </is>
-      </c>
-      <c r="C61" s="35" t="inlineStr">
-        <is>
-          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="34" t="inlineStr">
-        <is>
-          <t>Trường dùng chung</t>
-        </is>
-      </c>
-      <c r="B62" s="35" t="inlineStr">
-        <is>
-          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
-        </is>
-      </c>
-      <c r="C62" s="35" t="inlineStr">
-        <is>
-          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="34" t="inlineStr">
-        <is>
-          <t>Định dạng chữ</t>
-        </is>
-      </c>
-      <c r="B63" s="35" t="inlineStr">
-        <is>
           <t>Mỗi vị trí trong Word giữ nguyên đậm / nghiêng / in hoa / căn lề của bản gốc, kể cả khi dùng chung một trường. Phần mềm chỉ thay chữ, không đụng tới định dạng.</t>
         </is>
       </c>
-      <c r="C63" s="35" t="inlineStr">
-        <is>
-          <t>Mỗi vị trí trong Word giữ nguyên đậm / nghiêng / in hoa / căn lề của bản gốc, kể cả khi dùng chung một trường. Phần mềm chỉ thay chữ, không đụng tới định dạng.</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="61" ht="30" customHeight="1"/>
+    <row r="62" ht="30" customHeight="1"/>
+    <row r="63" ht="30" customHeight="1"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A1:B49"/>

</xml_diff>

<commit_message>
v1.6: Auto session restore, toast notifications, keyboard shortcuts, topbar order swapped, clean 2-row sidebar uploader, compact tab auto-expand
</commit_message>
<xml_diff>
--- a/sample/DULIEU_BaiGiang.xlsx
+++ b/sample/DULIEU_BaiGiang.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu bài giảng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dữ liệu bài giảng" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dữ liệu bài giảng'!$A$1:$B$49</definedName>
@@ -1326,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y60"/>
+  <dimension ref="A1:Y48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3194,183 +3194,15 @@
       <c r="Y48" s="111" t="n"/>
     </row>
     <row r="49" thickBot="1"/>
-    <row r="50">
-      <c r="A50" s="33" t="inlineStr">
-        <is>
-          <t>HƯỚNG DẪN NHẬP LIỆU</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="34" t="inlineStr">
-        <is>
-          <t>Bố cục bảng</t>
-        </is>
-      </c>
-      <c r="B51" s="35" t="inlineStr">
-        <is>
-          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
-        </is>
-      </c>
-      <c r="C51" s="35" t="inlineStr">
-        <is>
-          <t>Chia thành 7 khối, ngăn nhau bằng đường kẻ đậm, mỗi khối một màu ở cột A: xám = thông tin chung, hồng = người phê duyệt, tím = người thông qua, xanh ngọc = người biên soạn, xanh lá = Phần I, cam = Phần II, xanh dương = Phần III.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="45" customHeight="1">
-      <c r="A52" s="34" t="inlineStr">
-        <is>
-          <t>Cột A</t>
-        </is>
-      </c>
-      <c r="B52" s="35" t="inlineStr">
-        <is>
-          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
-        </is>
-      </c>
-      <c r="C52" s="35" t="inlineStr">
-        <is>
-          <t>Giữ nguyên, không sửa. Mỗi tên trường ứng với một chỗ {{...}} trong file Word mẫu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="34" t="inlineStr">
-        <is>
-          <t>Cột B</t>
-        </is>
-      </c>
-      <c r="B53" s="35" t="inlineStr">
-        <is>
-          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
-        </is>
-      </c>
-      <c r="C53" s="35" t="inlineStr">
-        <is>
-          <t>Chỉ sửa ở đây. Màu nền cho biết kiểu nhập: vàng = một dòng, xanh dương = nhiều dòng, cam = ngày tháng, xanh lá = số phút.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="34" t="inlineStr">
-        <is>
-          <t>Ô nhiều dòng</t>
-        </is>
-      </c>
-      <c r="B54" s="35" t="inlineStr">
-        <is>
-          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
-        </is>
-      </c>
-      <c r="C54" s="35" t="inlineStr">
-        <is>
-          <t>Bấm Alt + Enter để xuống dòng trong ô, mỗi gạch đầu dòng một dòng. Chiều cao dòng tự giãn theo nội dung, bề rộng cột cố định.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="34" t="inlineStr">
-        <is>
-          <t>Ô ngày tháng</t>
-        </is>
-      </c>
-      <c r="B55" s="35" t="inlineStr">
-        <is>
-          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
-        </is>
-      </c>
-      <c r="C55" s="35" t="inlineStr">
-        <is>
-          <t>Nhập dạng ngày/tháng/năm, ví dụ 07/04/2026. Ô đã khóa kiểu ngày, gõ sai Excel báo lỗi ngay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="34" t="inlineStr">
-        <is>
-          <t>Cú pháp mẫu Word</t>
-        </is>
-      </c>
-      <c r="B56" s="35" t="inlineStr">
-        <is>
-          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
-        </is>
-      </c>
-      <c r="C56" s="35" t="inlineStr">
-        <is>
-          <t>Chỗ ngày ghi là {{Tên trường:định dạng}}, ví dụ {{Ngày phê duyệt:Ngày dd tháng m năm yyyy}}. Tên trường là phần TRƯỚC dấu hai chấm, khớp với cột A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="34" t="inlineStr">
-        <is>
-          <t>Ký hiệu định dạng</t>
-        </is>
-      </c>
-      <c r="B57" s="35" t="inlineStr">
-        <is>
-          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
-        </is>
-      </c>
-      <c r="C57" s="35" t="inlineStr">
-        <is>
-          <t>dd = ngày, thêm số 0 nếu nhỏ hơn 10.   m = tháng, thêm số 0 nếu là tháng 1 hoặc 2, còn lại giữ nguyên (Nghị định 30/2020/NĐ-CP).   yyyy = năm 4 chữ số.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="34" t="inlineStr">
-        <is>
-          <t>Trang bìa</t>
-        </is>
-      </c>
-      <c r="B58" s="35" t="inlineStr">
-        <is>
-          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
-        </is>
-      </c>
-      <c r="C58" s="35" t="inlineStr">
-        <is>
-          <t>Không có trường riêng. Bìa ghi {{Ngày biên soạn:THÁNG m NĂM yyyy}}, phần mềm tự lấy tháng và năm của Ngày biên soạn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="34" t="inlineStr">
-        <is>
-          <t>Trường dùng chung</t>
-        </is>
-      </c>
-      <c r="B59" s="35" t="inlineStr">
-        <is>
-          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
-        </is>
-      </c>
-      <c r="C59" s="35" t="inlineStr">
-        <is>
-          <t>Tên học phần, Tên bài giảng, ba mốc ngày và ba nhóm nhân sự xuất hiện ở nhiều chỗ trong Word nhưng chỉ nhập một lần tại đây.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="34" t="inlineStr">
-        <is>
-          <t>Định dạng chữ</t>
-        </is>
-      </c>
-      <c r="B60" s="35" t="inlineStr">
-        <is>
-          <t>Mỗi vị trí trong Word giữ nguyên đậm / nghiêng / in hoa / căn lề của bản gốc, kể cả khi dùng chung một trường. Phần mềm chỉ thay chữ, không đụng tới định dạng.</t>
-        </is>
-      </c>
-      <c r="C60" s="35" t="inlineStr">
-        <is>
-          <t>Mỗi vị trí trong Word giữ nguyên đậm / nghiêng / in hoa / căn lề của bản gốc, kể cả khi dùng chung một trường. Phần mềm chỉ thay chữ, không đụng tới định dạng.</t>
-        </is>
-      </c>
-    </row>
+    <row r="52" ht="45" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="30" customHeight="1"/>
+    <row r="55" ht="30" customHeight="1"/>
+    <row r="56" ht="30" customHeight="1"/>
+    <row r="57" ht="30" customHeight="1"/>
+    <row r="58" ht="30" customHeight="1"/>
+    <row r="59" ht="30" customHeight="1"/>
+    <row r="60" ht="30" customHeight="1"/>
     <row r="61" ht="30" customHeight="1"/>
     <row r="62" ht="30" customHeight="1"/>
     <row r="63" ht="30" customHeight="1"/>

</xml_diff>